<commit_message>
Update morphometrics - tross.xlsx
</commit_message>
<xml_diff>
--- a/morphometrics/02_data/morphometrics - tross.xlsx
+++ b/morphometrics/02_data/morphometrics - tross.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mattg\Desktop\github\PSMFC-mytilus-byssus-pilot\morphometrics\02_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofwa-my.sharepoint.com/personal/matthew_george_dfw_wa_gov/Documents/Desktop/Github/PSMFC-mytilus-byssus-pilot/morphometrics/02_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44A61C96-9D5D-4DC5-A707-8F78B46E5AB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{44A61C96-9D5D-4DC5-A707-8F78B46E5AB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64DF6BD6-929C-46DE-852B-AF59E4B454CD}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{304823C0-04AF-47DA-8C98-4C863644367A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{304823C0-04AF-47DA-8C98-4C863644367A}"/>
   </bookViews>
   <sheets>
     <sheet name="mussels-all" sheetId="4" r:id="rId1"/>
@@ -25,12 +25,23 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2198" uniqueCount="441">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2186" uniqueCount="440">
   <si>
     <t>sdate</t>
   </si>
@@ -1350,9 +1361,6 @@
   </si>
   <si>
     <t>days_in_trt</t>
-  </si>
-  <si>
-    <t>2hr</t>
   </si>
 </sst>
 </file>
@@ -1455,9 +1463,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1495,7 +1503,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1601,7 +1609,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1743,7 +1751,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1823,8 +1831,8 @@
       <c r="D2" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>440</v>
+      <c r="E2" s="1">
+        <v>0</v>
       </c>
       <c r="F2" s="2">
         <v>44491</v>
@@ -1865,8 +1873,8 @@
       <c r="D3" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>440</v>
+      <c r="E3" s="1">
+        <v>0</v>
       </c>
       <c r="F3" s="2">
         <v>44491</v>
@@ -1907,8 +1915,8 @@
       <c r="D4" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>440</v>
+      <c r="E4" s="1">
+        <v>0</v>
       </c>
       <c r="F4" s="2">
         <v>44491</v>
@@ -1949,8 +1957,8 @@
       <c r="D5" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>440</v>
+      <c r="E5" s="1">
+        <v>0</v>
       </c>
       <c r="F5" s="2">
         <v>44491</v>
@@ -1991,8 +1999,8 @@
       <c r="D6" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>440</v>
+      <c r="E6" s="1">
+        <v>0</v>
       </c>
       <c r="F6" s="2">
         <v>44491</v>
@@ -2033,8 +2041,8 @@
       <c r="D7" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>440</v>
+      <c r="E7" s="1">
+        <v>0</v>
       </c>
       <c r="F7" s="2">
         <v>44491</v>
@@ -2075,8 +2083,8 @@
       <c r="D8" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>440</v>
+      <c r="E8" s="1">
+        <v>0</v>
       </c>
       <c r="F8" s="2">
         <v>44491</v>
@@ -2117,8 +2125,8 @@
       <c r="D9" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="E9" s="1" t="s">
-        <v>440</v>
+      <c r="E9" s="1">
+        <v>0</v>
       </c>
       <c r="F9" s="2">
         <v>44491</v>
@@ -2159,8 +2167,8 @@
       <c r="D10" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>440</v>
+      <c r="E10" s="1">
+        <v>0</v>
       </c>
       <c r="F10" s="2">
         <v>44491</v>
@@ -2201,8 +2209,8 @@
       <c r="D11" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>440</v>
+      <c r="E11" s="1">
+        <v>0</v>
       </c>
       <c r="F11" s="2">
         <v>44491</v>
@@ -2243,8 +2251,8 @@
       <c r="D12" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>440</v>
+      <c r="E12" s="1">
+        <v>0</v>
       </c>
       <c r="F12" s="2">
         <v>44491</v>
@@ -2285,8 +2293,8 @@
       <c r="D13" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>440</v>
+      <c r="E13" s="1">
+        <v>0</v>
       </c>
       <c r="F13" s="2">
         <v>44491</v>
@@ -2328,7 +2336,7 @@
         <v>10</v>
       </c>
       <c r="E14" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" s="2"/>
       <c r="G14" s="3">
@@ -2365,7 +2373,7 @@
         <v>10</v>
       </c>
       <c r="E15" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G15" s="3">
         <v>59</v>
@@ -2401,7 +2409,7 @@
         <v>10</v>
       </c>
       <c r="E16" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16" s="3">
         <v>66</v>
@@ -2437,7 +2445,7 @@
         <v>10</v>
       </c>
       <c r="E17" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G17" s="3">
         <v>57</v>
@@ -2473,7 +2481,7 @@
         <v>10</v>
       </c>
       <c r="E18" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18" s="3">
         <v>68</v>
@@ -2509,7 +2517,7 @@
         <v>11</v>
       </c>
       <c r="E19" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19" s="3">
         <v>57</v>
@@ -2545,7 +2553,7 @@
         <v>11</v>
       </c>
       <c r="E20" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G20" s="3">
         <v>52</v>
@@ -2581,7 +2589,7 @@
         <v>12</v>
       </c>
       <c r="E21" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G21" s="3">
         <v>62</v>
@@ -2617,7 +2625,7 @@
         <v>12</v>
       </c>
       <c r="E22" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G22" s="3">
         <v>52</v>
@@ -2653,7 +2661,7 @@
         <v>12</v>
       </c>
       <c r="E23" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" s="3">
         <v>56</v>
@@ -2689,7 +2697,7 @@
         <v>12</v>
       </c>
       <c r="E24" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G24" s="3">
         <v>63</v>
@@ -2725,7 +2733,7 @@
         <v>12</v>
       </c>
       <c r="E25" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G25" s="3">
         <v>60</v>
@@ -2761,7 +2769,7 @@
         <v>12</v>
       </c>
       <c r="E26" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G26" s="3">
         <v>58</v>
@@ -2797,7 +2805,7 @@
         <v>12</v>
       </c>
       <c r="E27" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G27" s="3">
         <v>57</v>
@@ -2833,7 +2841,7 @@
         <v>10</v>
       </c>
       <c r="E28" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F28" s="2">
         <v>44496</v>
@@ -2869,7 +2877,7 @@
         <v>10</v>
       </c>
       <c r="E29" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F29" s="2">
         <v>44496</v>
@@ -2905,7 +2913,7 @@
         <v>10</v>
       </c>
       <c r="E30" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F30" s="2">
         <v>44496</v>
@@ -2941,7 +2949,7 @@
         <v>10</v>
       </c>
       <c r="E31" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F31" s="2">
         <v>44496</v>
@@ -2977,7 +2985,7 @@
         <v>10</v>
       </c>
       <c r="E32" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F32" s="2">
         <v>44496</v>
@@ -3013,7 +3021,7 @@
         <v>11</v>
       </c>
       <c r="E33" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F33" s="2">
         <v>44498</v>
@@ -3049,7 +3057,7 @@
         <v>11</v>
       </c>
       <c r="E34" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F34" s="2">
         <v>44498</v>
@@ -3085,7 +3093,7 @@
         <v>11</v>
       </c>
       <c r="E35" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F35" s="2">
         <v>44498</v>
@@ -3121,7 +3129,7 @@
         <v>11</v>
       </c>
       <c r="E36" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F36" s="2">
         <v>44498</v>
@@ -3157,7 +3165,7 @@
         <v>11</v>
       </c>
       <c r="E37" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F37" s="2">
         <v>44498</v>
@@ -3193,7 +3201,7 @@
         <v>12</v>
       </c>
       <c r="E38" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F38" s="2">
         <v>44496</v>
@@ -3229,7 +3237,7 @@
         <v>12</v>
       </c>
       <c r="E39" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F39" s="2">
         <v>44496</v>
@@ -3265,7 +3273,7 @@
         <v>12</v>
       </c>
       <c r="E40" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F40" s="2">
         <v>44496</v>
@@ -3301,7 +3309,7 @@
         <v>12</v>
       </c>
       <c r="E41" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F41" s="2">
         <v>44496</v>
@@ -3337,7 +3345,7 @@
         <v>12</v>
       </c>
       <c r="E42" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F42" s="2">
         <v>44496</v>
@@ -5614,7 +5622,7 @@
         <v>19</v>
       </c>
       <c r="J98" s="3">
-        <f t="shared" ref="J98:J129" si="3">ROUND((4/3)*(G98/10)*(H98/10)*(I98/10),0)</f>
+        <f t="shared" ref="J98:J120" si="3">ROUND((4/3)*(G98/10)*(H98/10)*(I98/10),0)</f>
         <v>44</v>
       </c>
       <c r="M98" s="1" t="s">
@@ -6538,9 +6546,9 @@
         <f>VLOOKUP(C2,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="5">
         <f>VLOOKUP(C2,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I2" s="5">
         <v>122</v>
@@ -6591,9 +6599,9 @@
         <f>VLOOKUP(C3,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H3" s="5" t="str">
+      <c r="H3" s="5">
         <f>VLOOKUP(C3,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I3" s="9">
         <v>158</v>
@@ -6644,9 +6652,9 @@
         <f>VLOOKUP(C4,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H4" s="5" t="str">
+      <c r="H4" s="5">
         <f>VLOOKUP(C4,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I4" s="9">
         <v>28</v>
@@ -6697,9 +6705,9 @@
         <f>VLOOKUP(C5,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H5" s="5" t="str">
+      <c r="H5" s="5">
         <f>VLOOKUP(C5,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I5" s="5">
         <v>166</v>
@@ -6750,9 +6758,9 @@
         <f>VLOOKUP(C6,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H6" s="5" t="str">
+      <c r="H6" s="5">
         <f>VLOOKUP(C6,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I6" s="9">
         <v>92</v>
@@ -6803,9 +6811,9 @@
         <f>VLOOKUP(C7,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H7" s="5" t="str">
+      <c r="H7" s="5">
         <f>VLOOKUP(C7,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I7" s="9">
         <v>148</v>
@@ -6856,9 +6864,9 @@
         <f>VLOOKUP(C8,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H8" s="5" t="str">
+      <c r="H8" s="5">
         <f>VLOOKUP(C8,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I8" s="5">
         <v>186</v>
@@ -6909,9 +6917,9 @@
         <f>VLOOKUP(C9,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H9" s="5" t="str">
+      <c r="H9" s="5">
         <f>VLOOKUP(C9,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I9" s="9">
         <v>70.400000000000006</v>
@@ -6962,9 +6970,9 @@
         <f>VLOOKUP(C10,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H10" s="5" t="str">
+      <c r="H10" s="5">
         <f>VLOOKUP(C10,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I10" s="9">
         <v>65.400000000000006</v>
@@ -7015,9 +7023,9 @@
         <f>VLOOKUP(C11,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H11" s="5" t="str">
+      <c r="H11" s="5">
         <f>VLOOKUP(C11,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I11" s="5">
         <v>138</v>
@@ -7068,9 +7076,9 @@
         <f>VLOOKUP(C12,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H12" s="5" t="str">
+      <c r="H12" s="5">
         <f>VLOOKUP(C12,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I12" s="9">
         <v>44.4</v>
@@ -7121,9 +7129,9 @@
         <f>VLOOKUP(C13,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H13" s="5" t="str">
+      <c r="H13" s="5">
         <f>VLOOKUP(C13,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I13" s="9">
         <v>126</v>
@@ -7174,9 +7182,9 @@
         <f>VLOOKUP(C14,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H14" s="5" t="str">
+      <c r="H14" s="5">
         <f>VLOOKUP(C14,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I14" s="5">
         <v>136</v>
@@ -7227,9 +7235,9 @@
         <f>VLOOKUP(C15,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H15" s="5" t="str">
+      <c r="H15" s="5">
         <f>VLOOKUP(C15,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I15" s="9">
         <v>65.8</v>
@@ -7280,9 +7288,9 @@
         <f>VLOOKUP(C16,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H16" s="5" t="str">
+      <c r="H16" s="5">
         <f>VLOOKUP(C16,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I16" s="9">
         <v>160</v>
@@ -7333,9 +7341,9 @@
         <f>VLOOKUP(C17,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H17" s="5" t="str">
+      <c r="H17" s="5">
         <f>VLOOKUP(C17,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I17" s="5">
         <v>106</v>
@@ -7386,9 +7394,9 @@
         <f>VLOOKUP(C18,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H18" s="5" t="str">
+      <c r="H18" s="5">
         <f>VLOOKUP(C18,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I18" s="9">
         <v>95.2</v>
@@ -7439,9 +7447,9 @@
         <f>VLOOKUP(C19,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H19" s="5" t="str">
+      <c r="H19" s="5">
         <f>VLOOKUP(C19,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I19" s="9">
         <v>118</v>
@@ -7492,9 +7500,9 @@
         <f>VLOOKUP(C20,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H20" s="5" t="str">
+      <c r="H20" s="5">
         <f>VLOOKUP(C20,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I20" s="5">
         <v>27.6</v>
@@ -7545,9 +7553,9 @@
         <f>VLOOKUP(C21,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H21" s="5" t="str">
+      <c r="H21" s="5">
         <f>VLOOKUP(C21,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I21" s="5">
         <v>146</v>
@@ -7598,9 +7606,9 @@
         <f>VLOOKUP(C22,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H22" s="5" t="str">
+      <c r="H22" s="5">
         <f>VLOOKUP(C22,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I22" s="9">
         <v>106</v>
@@ -7651,9 +7659,9 @@
         <f>VLOOKUP(C23,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H23" s="5" t="str">
+      <c r="H23" s="5">
         <f>VLOOKUP(C23,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I23" s="5">
         <v>172</v>
@@ -7704,9 +7712,9 @@
         <f>VLOOKUP(C24,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H24" s="5" t="str">
+      <c r="H24" s="5">
         <f>VLOOKUP(C24,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I24" s="9">
         <v>66.400000000000006</v>
@@ -7757,9 +7765,9 @@
         <f>VLOOKUP(C25,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H25" s="5" t="str">
+      <c r="H25" s="5">
         <f>VLOOKUP(C25,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I25" s="9">
         <v>132</v>
@@ -7810,9 +7818,9 @@
         <f>VLOOKUP(C26,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H26" s="5" t="str">
+      <c r="H26" s="5">
         <f>VLOOKUP(C26,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I26" s="5">
         <v>174</v>
@@ -7863,9 +7871,9 @@
         <f>VLOOKUP(C27,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H27" s="5" t="str">
+      <c r="H27" s="5">
         <f>VLOOKUP(C27,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I27" s="9">
         <v>114</v>
@@ -7916,9 +7924,9 @@
         <f>VLOOKUP(C28,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H28" s="5" t="str">
+      <c r="H28" s="5">
         <f>VLOOKUP(C28,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I28" s="9">
         <v>130</v>
@@ -7969,9 +7977,9 @@
         <f>VLOOKUP(C29,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H29" s="5" t="str">
+      <c r="H29" s="5">
         <f>VLOOKUP(C29,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I29" s="5">
         <v>188</v>
@@ -8022,9 +8030,9 @@
         <f>VLOOKUP(C30,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H30" s="5" t="str">
+      <c r="H30" s="5">
         <f>VLOOKUP(C30,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I30" s="9">
         <v>74.2</v>
@@ -8075,9 +8083,9 @@
         <f>VLOOKUP(C31,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H31" s="5" t="str">
+      <c r="H31" s="5">
         <f>VLOOKUP(C31,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I31" s="9">
         <v>85.6</v>
@@ -8128,9 +8136,9 @@
         <f>VLOOKUP(C32,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H32" s="5" t="str">
+      <c r="H32" s="5">
         <f>VLOOKUP(C32,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I32" s="5">
         <v>116</v>
@@ -8181,9 +8189,9 @@
         <f>VLOOKUP(C33,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H33" s="5" t="str">
+      <c r="H33" s="5">
         <f>VLOOKUP(C33,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I33" s="9">
         <v>138</v>
@@ -8234,9 +8242,9 @@
         <f>VLOOKUP(C34,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H34" s="5" t="str">
+      <c r="H34" s="5">
         <f>VLOOKUP(C34,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I34" s="9">
         <v>112</v>
@@ -8817,9 +8825,9 @@
         <f>VLOOKUP(C45,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H45" s="5" t="str">
+      <c r="H45" s="5">
         <f>VLOOKUP(C45,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I45" s="5">
         <v>132</v>
@@ -8870,9 +8878,9 @@
         <f>VLOOKUP(C46,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H46" s="5" t="str">
+      <c r="H46" s="5">
         <f>VLOOKUP(C46,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I46" s="9">
         <v>152</v>
@@ -8923,9 +8931,9 @@
         <f>VLOOKUP(C47,'mussels-all'!B:D,3,FALSE)</f>
         <v>lab_control</v>
       </c>
-      <c r="H47" s="5" t="str">
+      <c r="H47" s="5">
         <f>VLOOKUP(C47,'mussels-all'!B:E,4,FALSE)</f>
-        <v>2hr</v>
+        <v>0</v>
       </c>
       <c r="I47" s="9">
         <v>132</v>
@@ -19231,4 +19239,10 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{45011977-b912-4387-97a4-f4c94a801377}" enabled="1" method="Standard" siteId="{11d0e217-264e-400a-8ba0-57dcc127d72d}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>